<commit_message>
New results wte with Lukas capex definition
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/MEA/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/MEA/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2230,6 +2230,521 @@
       <c r="AE17" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\MEA\20260128180958_dh_ratio_1_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>10630997.08808911</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3971300.937581479</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3291398.029133782</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3606118.490387282</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7577419.427968761</v>
+      </c>
+      <c r="G18" t="n">
+        <v>3291398.029133782</v>
+      </c>
+      <c r="H18" t="n">
+        <v>12583.08977498814</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-3668293.219629269</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3417889.760840844</v>
+      </c>
+      <c r="M18" t="n">
+        <v>10630997.08808911</v>
+      </c>
+      <c r="N18" t="n">
+        <v>22788.31043805332</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>22788.31043805332</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>22785.93173893896</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>2.378699114368705</v>
+      </c>
+      <c r="V18" t="n">
+        <v>7.209000110626221</v>
+      </c>
+      <c r="W18" t="n">
+        <v>10630997.08808911</v>
+      </c>
+      <c r="X18" t="n">
+        <v>10630997.08808911</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>dh_ratio_0_costs</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\MEA\20260303113549_dh_ratio_0_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>11472878.98551224</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3971300.937581479</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3291398.029133782</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3606118.490387282</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>7577419.427968761</v>
+      </c>
+      <c r="G19" t="n">
+        <v>3291398.029133782</v>
+      </c>
+      <c r="H19" t="n">
+        <v>35945.8881588577</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-2865982.061968812</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>3434097.702219653</v>
+      </c>
+      <c r="M19" t="n">
+        <v>11472878.98551224</v>
+      </c>
+      <c r="N19" t="n">
+        <v>22896.36338057872</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>22896.36338057872</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>22893.98468146435</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="n">
+        <v>2.378699114368705</v>
+      </c>
+      <c r="V19" t="n">
+        <v>7.083999872207642</v>
+      </c>
+      <c r="W19" t="n">
+        <v>11472878.98551224</v>
+      </c>
+      <c r="X19" t="n">
+        <v>11472878.98551224</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>dh_ratio_0.25_costs</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\MEA\20260303113807_dh_ratio_0.25_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>12765616.06738241</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3966641.260460024</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3289208.746615126</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3603171.236910735</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>7569812.497370759</v>
+      </c>
+      <c r="G20" t="n">
+        <v>3289208.746615126</v>
+      </c>
+      <c r="H20" t="n">
+        <v>547797.4516861945</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-2445827.708458884</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3804625.080169213</v>
+      </c>
+      <c r="M20" t="n">
+        <v>12765616.06738241</v>
+      </c>
+      <c r="N20" t="n">
+        <v>25366.54461437949</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>25366.54461437949</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>25364.16720112809</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>2.377413251389333</v>
+      </c>
+      <c r="V20" t="n">
+        <v>8.136000156402588</v>
+      </c>
+      <c r="W20" t="n">
+        <v>12765616.06738241</v>
+      </c>
+      <c r="X20" t="n">
+        <v>12765616.06738241</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>dh_ratio_0.5_costs</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\MEA\20260303114031_dh_ratio_0.5_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>14356301.02713308</v>
+      </c>
+      <c r="B21" t="n">
+        <v>3962577.690295069</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3287299.536407297</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3600578.433583683</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>7563156.123878751</v>
+      </c>
+      <c r="G21" t="n">
+        <v>3287299.536407297</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1391991.937409291</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-2290352.096638842</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>4404205.526076586</v>
+      </c>
+      <c r="M21" t="n">
+        <v>14356301.02713308</v>
+      </c>
+      <c r="N21" t="n">
+        <v>29363.74642705184</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>29363.74642705184</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>29361.3701738439</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>2.376253207936251</v>
+      </c>
+      <c r="V21" t="n">
+        <v>8.167999982833862</v>
+      </c>
+      <c r="W21" t="n">
+        <v>14356301.02713308</v>
+      </c>
+      <c r="X21" t="n">
+        <v>14356301.02713308</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>dh_ratio_0.75_costs</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\MEA\20260303114241_dh_ratio_0.75_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>16047219.00953853</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3960083.715782794</v>
+      </c>
+      <c r="C22" t="n">
+        <v>3286127.778223333</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3598976.306195484</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>7559060.021978278</v>
+      </c>
+      <c r="G22" t="n">
+        <v>3286127.778223333</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2338001.787695138</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-2205236.36615914</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>5069265.787800925</v>
+      </c>
+      <c r="M22" t="n">
+        <v>16047219.00953853</v>
+      </c>
+      <c r="N22" t="n">
+        <v>33797.4807747201</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>33797.4807747201</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>33795.10525200616</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>2.375522713928874</v>
+      </c>
+      <c r="V22" t="n">
+        <v>7.789000034332275</v>
+      </c>
+      <c r="W22" t="n">
+        <v>16047219.00953853</v>
+      </c>
+      <c r="X22" t="n">
+        <v>16047219.00953853</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>dh_ratio_1_costs</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\MEA\20260303114521_dh_ratio_1_costs</t>
         </is>
       </c>
     </row>

</xml_diff>